<commit_message>
one excel was opened when commit, refreshing commit
</commit_message>
<xml_diff>
--- a/figures/TCAD_Refaldi_calibration_progress.xlsx
+++ b/figures/TCAD_Refaldi_calibration_progress.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshs\Desktop\local-laptop\EDLtarget-manuscript-Mar\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4C70D07-5D9A-470D-AC79-DF5D3073D3DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{606A91E5-8770-47E3-9787-A5D1401DED52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -741,8 +741,8 @@
         <v>3.8960000000000002E-2</v>
       </c>
       <c r="G2">
-        <f>1.2+F2/15*0.1</f>
-        <v>1.2002597333333334</v>
+        <f>F2*0.1/5/1.5*1.1-0.015</f>
+        <v>-1.4428586666666667E-2</v>
       </c>
       <c r="H2">
         <v>1E-4</v>
@@ -751,8 +751,8 @@
         <v>-7.7920000000000003E-2</v>
       </c>
       <c r="J2">
-        <f>1.2+I2/15*0.1</f>
-        <v>1.1994805333333334</v>
+        <f>I2*0.1/5/1.5*1.1-0.015</f>
+        <v>-1.6142826666666665E-2</v>
       </c>
       <c r="M2" s="1">
         <v>2.4999999999999999E-13</v>
@@ -861,8 +861,8 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <f t="shared" ref="G3:G35" si="3">1.2+F3/15*0.1</f>
-        <v>1.2</v>
+        <f t="shared" ref="G3:G35" si="3">F3*0.1/5/1.5*1.1-0.015</f>
+        <v>-1.4999999999999999E-2</v>
       </c>
       <c r="H3">
         <v>1.8000000000000001E-4</v>
@@ -871,8 +871,8 @@
         <v>-7.7920000000000003E-2</v>
       </c>
       <c r="J3">
-        <f t="shared" ref="J3:J39" si="4">1.2+I3/15*0.1</f>
-        <v>1.1994805333333334</v>
+        <f t="shared" ref="J3:J39" si="4">I3*0.1/5/1.5*1.1-0.015</f>
+        <v>-1.6142826666666665E-2</v>
       </c>
       <c r="M3" s="1">
         <v>7.5000000000000004E-13</v>
@@ -980,7 +980,7 @@
       </c>
       <c r="G4">
         <f t="shared" si="3"/>
-        <v>1.1998701333333333</v>
+        <v>-1.5285706666666666E-2</v>
       </c>
       <c r="H4">
         <v>3.4000000000000002E-4</v>
@@ -990,7 +990,7 @@
       </c>
       <c r="J4">
         <f t="shared" si="4"/>
-        <v>1.1993506666666667</v>
+        <v>-1.6428533333333332E-2</v>
       </c>
       <c r="M4" s="1">
         <v>9.9999999999999998E-13</v>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="G5">
         <f t="shared" si="3"/>
-        <v>1.2003896000000001</v>
+        <v>-1.414288E-2</v>
       </c>
       <c r="H5">
         <v>5.8E-4</v>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="J5">
         <f t="shared" si="4"/>
-        <v>1.1997402666666666</v>
+        <v>-1.5571413333333332E-2</v>
       </c>
       <c r="M5" s="1">
         <v>2E-12</v>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="G6">
         <f t="shared" si="3"/>
-        <v>1.1998701333333333</v>
+        <v>-1.5285706666666666E-2</v>
       </c>
       <c r="H6">
         <v>1.08E-3</v>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="J6">
         <f t="shared" si="4"/>
-        <v>1.1997402666666666</v>
+        <v>-1.5571413333333332E-2</v>
       </c>
       <c r="M6" s="1">
         <v>3.9999999999999999E-12</v>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="G7">
         <f t="shared" si="3"/>
-        <v>1.2002597333333334</v>
+        <v>-1.4428586666666667E-2</v>
       </c>
       <c r="H7">
         <v>1.81E-3</v>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="J7">
         <f t="shared" si="4"/>
-        <v>1.1994805333333334</v>
+        <v>-1.6142826666666665E-2</v>
       </c>
       <c r="M7" s="1">
         <v>7.9999999999999998E-12</v>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="G8">
         <f t="shared" si="3"/>
-        <v>1.2002597333333334</v>
+        <v>-1.4428586666666667E-2</v>
       </c>
       <c r="H8">
         <v>3.2100000000000002E-3</v>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="J8">
         <f t="shared" si="4"/>
-        <v>1.1993506666666667</v>
+        <v>-1.6428533333333332E-2</v>
       </c>
       <c r="M8" s="1">
         <v>9.9999999999999994E-12</v>
@@ -1565,7 +1565,7 @@
       </c>
       <c r="G9">
         <f t="shared" si="3"/>
-        <v>1.2003896000000001</v>
+        <v>-1.414288E-2</v>
       </c>
       <c r="H9">
         <v>5.6899999999999997E-3</v>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="J9">
         <f t="shared" si="4"/>
-        <v>1.1990909333333333</v>
+        <v>-1.6999946666666668E-2</v>
       </c>
       <c r="M9" s="1">
         <v>1.7999999999999999E-11</v>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="G10">
         <f t="shared" si="3"/>
-        <v>1.2001298666666667</v>
+        <v>-1.4714293333333333E-2</v>
       </c>
       <c r="H10">
         <v>1.047E-2</v>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="J10">
         <f t="shared" si="4"/>
-        <v>1.1988311999999999</v>
+        <v>-1.7571360000000001E-2</v>
       </c>
       <c r="M10" s="1">
         <v>3.3999999999999999E-11</v>
@@ -1799,7 +1799,7 @@
       </c>
       <c r="G11">
         <f t="shared" si="3"/>
-        <v>1.2</v>
+        <v>-1.4999999999999999E-2</v>
       </c>
       <c r="H11">
         <v>1.8239999999999999E-2</v>
@@ -1809,7 +1809,7 @@
       </c>
       <c r="J11">
         <f t="shared" si="4"/>
-        <v>1.1981818</v>
+        <v>-1.9000039999999999E-2</v>
       </c>
       <c r="M11" s="1">
         <v>6.6000000000000005E-11</v>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="G12">
         <f t="shared" si="3"/>
-        <v>1.1993506666666667</v>
+        <v>-1.6428533333333332E-2</v>
       </c>
       <c r="H12">
         <v>3.236E-2</v>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="J12">
         <f t="shared" si="4"/>
-        <v>1.1971428666666666</v>
+        <v>-2.1285693333333335E-2</v>
       </c>
       <c r="M12" s="1">
         <v>1E-10</v>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="G13">
         <f t="shared" si="3"/>
-        <v>1.1992208</v>
+        <v>-1.6714239999999998E-2</v>
       </c>
       <c r="H13">
         <v>6.0690000000000001E-2</v>
@@ -2043,7 +2043,7 @@
       </c>
       <c r="J13">
         <f t="shared" si="4"/>
-        <v>1.1967532666666667</v>
+        <v>-2.2142813333333334E-2</v>
       </c>
       <c r="M13" s="1">
         <v>2.0751743999999999E-10</v>
@@ -2150,7 +2150,7 @@
       </c>
       <c r="G14">
         <f t="shared" si="3"/>
-        <v>1.1989610666666666</v>
+        <v>-1.7285653333333335E-2</v>
       </c>
       <c r="H14">
         <v>0.10571</v>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="J14">
         <f t="shared" si="4"/>
-        <v>1.1959739999999999</v>
+        <v>-2.3857200000000002E-2</v>
       </c>
       <c r="M14" s="1">
         <v>4.2255232E-10</v>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="G15">
         <f t="shared" si="3"/>
-        <v>1.1989610666666666</v>
+        <v>-1.7285653333333335E-2</v>
       </c>
       <c r="H15">
         <v>0.19461000000000001</v>
@@ -2277,7 +2277,7 @@
       </c>
       <c r="J15">
         <f t="shared" si="4"/>
-        <v>1.1953246666666666</v>
+        <v>-2.5285733333333338E-2</v>
       </c>
       <c r="M15" s="1">
         <v>8.5262207999999996E-10</v>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="G16">
         <f t="shared" si="3"/>
-        <v>1.1983116666666667</v>
+        <v>-1.8714333333333333E-2</v>
       </c>
       <c r="H16">
         <v>0.34527000000000002</v>
@@ -2394,7 +2394,7 @@
       </c>
       <c r="J16">
         <f t="shared" si="4"/>
-        <v>1.1942857333333332</v>
+        <v>-2.757138666666667E-2</v>
       </c>
       <c r="M16" s="1">
         <v>1.0000000000000001E-9</v>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="G17">
         <f t="shared" si="3"/>
-        <v>1.1977921999999999</v>
+        <v>-1.9857159999999999E-2</v>
       </c>
       <c r="H17">
         <v>0.59031999999999996</v>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="J17">
         <f t="shared" si="4"/>
-        <v>1.1924675333333332</v>
+        <v>-3.1571426666666666E-2</v>
       </c>
       <c r="M17" s="1">
         <v>1.8601395E-9</v>
@@ -2618,7 +2618,7 @@
       </c>
       <c r="G18">
         <f t="shared" si="3"/>
-        <v>1.1967532666666667</v>
+        <v>-2.2142813333333334E-2</v>
       </c>
       <c r="H18">
         <v>1.04732</v>
@@ -2628,7 +2628,7 @@
       </c>
       <c r="J18">
         <f t="shared" si="4"/>
-        <v>1.1910389333333333</v>
+        <v>-3.4714346666666673E-2</v>
       </c>
       <c r="M18" s="1">
         <v>3.5804185999999999E-9</v>
@@ -2736,7 +2736,7 @@
       </c>
       <c r="G19">
         <f t="shared" si="3"/>
-        <v>1.1959739999999999</v>
+        <v>-2.3857200000000002E-2</v>
       </c>
       <c r="H19">
         <v>1.8928199999999999</v>
@@ -2746,7 +2746,7 @@
       </c>
       <c r="J19">
         <f t="shared" si="4"/>
-        <v>1.1889610666666666</v>
+        <v>-3.9285653333333337E-2</v>
       </c>
       <c r="M19" s="1">
         <v>7.0209766999999997E-9</v>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="G20">
         <f t="shared" si="3"/>
-        <v>1.1945454666666666</v>
+        <v>-2.6999973333333333E-2</v>
       </c>
       <c r="H20">
         <v>3.23624</v>
@@ -2864,7 +2864,7 @@
       </c>
       <c r="J20">
         <f t="shared" si="4"/>
-        <v>1.1874026</v>
+        <v>-4.2714280000000007E-2</v>
       </c>
       <c r="M20" s="1">
         <v>1E-8</v>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="G21">
         <f t="shared" si="3"/>
-        <v>1.192987</v>
+        <v>-3.04286E-2</v>
       </c>
       <c r="H21">
         <v>5.1385800000000001</v>
@@ -2982,7 +2982,7 @@
       </c>
       <c r="J21">
         <f t="shared" si="4"/>
-        <v>1.1844155999999999</v>
+        <v>-4.9285680000000012E-2</v>
       </c>
       <c r="M21" s="1">
         <v>1.6881116000000001E-8</v>
@@ -3090,7 +3090,7 @@
       </c>
       <c r="G22">
         <f t="shared" si="3"/>
-        <v>1.1907791999999999</v>
+        <v>-3.5285759999999999E-2</v>
       </c>
       <c r="H22">
         <v>9.1167400000000001</v>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="J22">
         <f t="shared" si="4"/>
-        <v>1.1819480666666666</v>
+        <v>-5.4714253333333344E-2</v>
       </c>
       <c r="M22" s="1">
         <v>3.0643349000000001E-8</v>
@@ -3208,7 +3208,7 @@
       </c>
       <c r="G23">
         <f t="shared" si="3"/>
-        <v>1.1870129999999999</v>
+        <v>-4.3571400000000003E-2</v>
       </c>
       <c r="H23">
         <v>16.174669999999999</v>
@@ -3218,7 +3218,7 @@
       </c>
       <c r="J23">
         <f t="shared" si="4"/>
-        <v>1.1790909333333333</v>
+        <v>-6.099994666666668E-2</v>
       </c>
       <c r="M23" s="1">
         <v>5.8167813000000005E-8</v>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="G24">
         <f t="shared" si="3"/>
-        <v>1.1841558666666667</v>
+        <v>-4.9857093333333338E-2</v>
       </c>
       <c r="H24">
         <v>28.696660000000001</v>
@@ -3336,7 +3336,7 @@
       </c>
       <c r="J24">
         <f t="shared" si="4"/>
-        <v>1.1757142666666667</v>
+        <v>-6.8428613333333346E-2</v>
       </c>
       <c r="M24" s="1">
         <v>9.9999999999999995E-8</v>
@@ -3444,7 +3444,7 @@
       </c>
       <c r="G25">
         <f t="shared" si="3"/>
-        <v>1.1812987333333334</v>
+        <v>-5.6142786666666673E-2</v>
       </c>
       <c r="H25">
         <v>39.298639999999999</v>
@@ -3454,7 +3454,7 @@
       </c>
       <c r="J25">
         <f t="shared" si="4"/>
-        <v>1.1731168666666667</v>
+        <v>-7.4142893333333348E-2</v>
       </c>
       <c r="M25" s="1">
         <v>1.9999999999999999E-7</v>
@@ -3562,7 +3562,7 @@
       </c>
       <c r="G26">
         <f t="shared" si="3"/>
-        <v>1.1759739999999999</v>
+        <v>-6.7857200000000006E-2</v>
       </c>
       <c r="H26">
         <v>69.722589999999997</v>
@@ -3572,7 +3572,7 @@
       </c>
       <c r="J26">
         <f t="shared" si="4"/>
-        <v>1.1690909333333332</v>
+        <v>-8.2999946666666671E-2</v>
       </c>
       <c r="M26" s="1">
         <v>4.2019572E-7</v>
@@ -3680,7 +3680,7 @@
       </c>
       <c r="G27">
         <f t="shared" si="3"/>
-        <v>1.1719480666666666</v>
+        <v>-7.6714253333333343E-2</v>
       </c>
       <c r="H27">
         <v>126.00901</v>
@@ -3690,7 +3690,7 @@
       </c>
       <c r="J27">
         <f t="shared" si="4"/>
-        <v>1.1650649333333334</v>
+        <v>-9.1857146666666667E-2</v>
       </c>
       <c r="M27" s="1">
         <v>8.6058715000000004E-7</v>
@@ -3798,7 +3798,7 @@
       </c>
       <c r="G28">
         <f t="shared" si="3"/>
-        <v>1.1675324666666667</v>
+        <v>-8.6428573333333342E-2</v>
       </c>
       <c r="H28">
         <v>227.73497</v>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="J28">
         <f t="shared" si="4"/>
-        <v>1.1606493333333332</v>
+        <v>-0.10157146666666667</v>
       </c>
       <c r="M28" s="1">
         <v>9.9999999999999995E-7</v>
@@ -3916,7 +3916,7 @@
       </c>
       <c r="G29">
         <f t="shared" si="3"/>
-        <v>1.1618181999999999</v>
+        <v>-9.8999959999999998E-2</v>
       </c>
       <c r="H29">
         <v>451.45916</v>
@@ -3926,7 +3926,7 @@
       </c>
       <c r="J29">
         <f t="shared" si="4"/>
-        <v>1.1528571333333333</v>
+        <v>-0.11871430666666669</v>
       </c>
       <c r="M29" s="1">
         <v>1.8807829000000001E-6</v>
@@ -4034,7 +4034,7 @@
       </c>
       <c r="G30">
         <f t="shared" si="3"/>
-        <v>1.1575324666666666</v>
+        <v>-0.10842857333333335</v>
       </c>
       <c r="H30">
         <v>800.96668999999997</v>
@@ -4044,7 +4044,7 @@
       </c>
       <c r="J30">
         <f t="shared" si="4"/>
-        <v>1.1476623333333333</v>
+        <v>-0.13014286666666669</v>
       </c>
       <c r="M30" s="1">
         <v>3.6423486E-6</v>
@@ -4152,7 +4152,7 @@
       </c>
       <c r="G31">
         <f t="shared" si="3"/>
-        <v>1.1535064666666666</v>
+        <v>-0.11728577333333334</v>
       </c>
       <c r="H31">
         <v>1447.57999</v>
@@ -4162,7 +4162,7 @@
       </c>
       <c r="J31">
         <f t="shared" si="4"/>
-        <v>1.1419480666666666</v>
+        <v>-0.14271425333333332</v>
       </c>
       <c r="M31" s="1">
         <v>7.1654801000000005E-6</v>
@@ -4270,7 +4270,7 @@
       </c>
       <c r="G32">
         <f t="shared" si="3"/>
-        <v>1.1471428666666665</v>
+        <v>-0.13128569333333334</v>
       </c>
       <c r="H32">
         <v>1875.3933400000001</v>
@@ -4280,7 +4280,7 @@
       </c>
       <c r="J32">
         <f t="shared" si="4"/>
-        <v>1.1381817999999999</v>
+        <v>-0.15100004</v>
       </c>
       <c r="M32" s="1">
         <v>1.0000000000000001E-5</v>
@@ -4388,7 +4388,7 @@
       </c>
       <c r="G33">
         <f t="shared" si="3"/>
-        <v>1.1427272666666666</v>
+        <v>-0.14100001333333334</v>
       </c>
       <c r="H33">
         <v>3266.30116</v>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="J33">
         <f t="shared" si="4"/>
-        <v>1.1328571333333333</v>
+        <v>-0.16271430666666664</v>
       </c>
       <c r="M33" s="1">
         <v>1.7046262999999999E-5</v>
@@ -4506,7 +4506,7 @@
       </c>
       <c r="G34">
         <f t="shared" si="3"/>
-        <v>1.1384415333333333</v>
+        <v>-0.15042862666666668</v>
       </c>
       <c r="H34">
         <v>5794.9835700000003</v>
@@ -4516,7 +4516,7 @@
       </c>
       <c r="J34">
         <f t="shared" si="4"/>
-        <v>1.1263636666666665</v>
+        <v>-0.17699993333333336</v>
       </c>
       <c r="M34" s="1">
         <v>3.1138788999999997E-5</v>
@@ -4624,7 +4624,7 @@
       </c>
       <c r="G35">
         <f t="shared" si="3"/>
-        <v>1.1348052</v>
+        <v>-0.15842856000000005</v>
       </c>
       <c r="H35">
         <v>10281.303809999999</v>
@@ -4634,7 +4634,7 @@
       </c>
       <c r="J35">
         <f t="shared" si="4"/>
-        <v>1.1205194666666667</v>
+        <v>-0.18985717333333335</v>
       </c>
       <c r="M35" s="1">
         <v>5.9323841000000002E-5</v>
@@ -4742,7 +4742,7 @@
       </c>
       <c r="J36">
         <f t="shared" si="4"/>
-        <v>1.1167532666666666</v>
+        <v>-0.19814281333333333</v>
       </c>
       <c r="M36">
         <v>1E-4</v>
@@ -4850,7 +4850,7 @@
       </c>
       <c r="J37">
         <f t="shared" si="4"/>
-        <v>1.1103896</v>
+        <v>-0.21214288000000003</v>
       </c>
       <c r="M37">
         <v>2.1274021E-4</v>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="J38">
         <f t="shared" si="4"/>
-        <v>1.1037662666666666</v>
+        <v>-0.22671421333333336</v>
       </c>
       <c r="M38">
         <v>4.3822062000000003E-4</v>
@@ -5066,7 +5066,7 @@
       </c>
       <c r="J39">
         <f t="shared" si="4"/>
-        <v>1.0966233999999999</v>
+        <v>-0.24242852000000004</v>
       </c>
       <c r="M39">
         <v>8.8918145E-4</v>

</xml_diff>